<commit_message>
[Nairne] Distributions tab: add Expected Gross + Weighted Expense columns
Per-Party Settlement section now shows the full earnings breakdown
for each party, not just the net:

  Party | Expected Gross | Weighted Expense | Expected Net | Cash Paid
  Out | Outstanding | Suggested Recipient | Status

Expected Gross + Weighted Expense both pull from Consultant Summary
via VLOOKUP (cols D and F). Expected Net is computed as Gross −
Weighted Expense. Outstanding = Net − Cash Paid Out. Totals at the
bottom sum each money column for the Armada GP Pool. TruQuant row
below the total shows its full breakdown too.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Armada_Consultant_Splits.xlsx
+++ b/Armada_Consultant_Splits.xlsx
@@ -6174,15 +6174,15 @@
   <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6428,25 +6428,35 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
+          <t>Expected Gross</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Weighted Expense</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
           <t>Expected Net</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Cash Paid Out</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Outstanding</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Suggested Recipient / Wire Info</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -6459,20 +6469,28 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>IFERROR(VLOOKUP(A27, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A27, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A27, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A27, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D27" s="10">
         <f>B27-C27</f>
         <v/>
       </c>
-      <c r="E27" s="28" t="inlineStr"/>
-      <c r="F27">
-        <f>IF(ROUND(D27,2)=0,"Settled",IF(ROUND(D27,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E27" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A27, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F27" s="10">
+        <f>D27-E27</f>
+        <v/>
+      </c>
+      <c r="G27" s="28" t="inlineStr"/>
+      <c r="H27">
+        <f>IF(ROUND(F27,2)=0,"Settled",IF(ROUND(F27,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6483,20 +6501,28 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>IFERROR(VLOOKUP(A28, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A28, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A28, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A28, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D28" s="10">
         <f>B28-C28</f>
         <v/>
       </c>
-      <c r="E28" s="28" t="inlineStr"/>
-      <c r="F28">
-        <f>IF(ROUND(D28,2)=0,"Settled",IF(ROUND(D28,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E28" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A28, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F28" s="10">
+        <f>D28-E28</f>
+        <v/>
+      </c>
+      <c r="G28" s="28" t="inlineStr"/>
+      <c r="H28">
+        <f>IF(ROUND(F28,2)=0,"Settled",IF(ROUND(F28,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6507,20 +6533,28 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>IFERROR(VLOOKUP(A29, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A29, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A29, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A29, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D29" s="10">
         <f>B29-C29</f>
         <v/>
       </c>
-      <c r="E29" s="28" t="inlineStr"/>
-      <c r="F29">
-        <f>IF(ROUND(D29,2)=0,"Settled",IF(ROUND(D29,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E29" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A29, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F29" s="10">
+        <f>D29-E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="28" t="inlineStr"/>
+      <c r="H29">
+        <f>IF(ROUND(F29,2)=0,"Settled",IF(ROUND(F29,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6531,20 +6565,28 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>IFERROR(VLOOKUP(A30, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A30, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A30, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A30, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D30" s="10">
         <f>B30-C30</f>
         <v/>
       </c>
-      <c r="E30" s="28" t="inlineStr"/>
-      <c r="F30">
-        <f>IF(ROUND(D30,2)=0,"Settled",IF(ROUND(D30,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E30" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A30, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F30" s="10">
+        <f>D30-E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="28" t="inlineStr"/>
+      <c r="H30">
+        <f>IF(ROUND(F30,2)=0,"Settled",IF(ROUND(F30,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6555,20 +6597,28 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>IFERROR(VLOOKUP(A31, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A31, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A31, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A31, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D31" s="10">
         <f>B31-C31</f>
         <v/>
       </c>
-      <c r="E31" s="28" t="inlineStr"/>
-      <c r="F31">
-        <f>IF(ROUND(D31,2)=0,"Settled",IF(ROUND(D31,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E31" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A31, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F31" s="10">
+        <f>D31-E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="28" t="inlineStr"/>
+      <c r="H31">
+        <f>IF(ROUND(F31,2)=0,"Settled",IF(ROUND(F31,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6579,20 +6629,28 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>IFERROR(VLOOKUP(A32, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A32, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A32, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A32, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D32" s="10">
         <f>B32-C32</f>
         <v/>
       </c>
-      <c r="E32" s="28" t="inlineStr"/>
-      <c r="F32">
-        <f>IF(ROUND(D32,2)=0,"Settled",IF(ROUND(D32,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E32" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A32, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F32" s="10">
+        <f>D32-E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="28" t="inlineStr"/>
+      <c r="H32">
+        <f>IF(ROUND(F32,2)=0,"Settled",IF(ROUND(F32,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6603,20 +6661,28 @@
         </is>
       </c>
       <c r="B33" s="10">
-        <f>IFERROR(VLOOKUP(A33, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A33, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C33" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A33, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A33, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D33" s="10">
         <f>B33-C33</f>
         <v/>
       </c>
-      <c r="E33" s="28" t="inlineStr"/>
-      <c r="F33">
-        <f>IF(ROUND(D33,2)=0,"Settled",IF(ROUND(D33,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E33" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A33, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F33" s="10">
+        <f>D33-E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="28" t="inlineStr"/>
+      <c r="H33">
+        <f>IF(ROUND(F33,2)=0,"Settled",IF(ROUND(F33,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6627,20 +6693,28 @@
         </is>
       </c>
       <c r="B34" s="10">
-        <f>IFERROR(VLOOKUP(A34, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A34, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C34" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A34, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A34, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D34" s="10">
         <f>B34-C34</f>
         <v/>
       </c>
-      <c r="E34" s="28" t="inlineStr"/>
-      <c r="F34">
-        <f>IF(ROUND(D34,2)=0,"Settled",IF(ROUND(D34,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E34" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A34, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F34" s="10">
+        <f>D34-E34</f>
+        <v/>
+      </c>
+      <c r="G34" s="28" t="inlineStr"/>
+      <c r="H34">
+        <f>IF(ROUND(F34,2)=0,"Settled",IF(ROUND(F34,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6651,20 +6725,28 @@
         </is>
       </c>
       <c r="B35" s="10">
-        <f>IFERROR(VLOOKUP(A35, 'Consultant Summary'!$A$2:$G$19, 7, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(A35, 'Consultant Summary'!$A$2:$G$19, 4, FALSE), 0)</f>
         <v/>
       </c>
       <c r="C35" s="10">
-        <f>SUMIFS(Dist_Amount, Dist_Party, A35, Dist_Type, "Payout")</f>
+        <f>IFERROR(VLOOKUP(A35, 'Consultant Summary'!$A$2:$G$19, 6, FALSE), 0)</f>
         <v/>
       </c>
       <c r="D35" s="10">
         <f>B35-C35</f>
         <v/>
       </c>
-      <c r="E35" s="28" t="inlineStr"/>
-      <c r="F35">
-        <f>IF(ROUND(D35,2)=0,"Settled",IF(ROUND(D35,2)&lt;0,"Overpaid","Outstanding"))</f>
+      <c r="E35" s="10">
+        <f>SUMIFS(Dist_Amount, Dist_Party, A35, Dist_Type, "Payout")</f>
+        <v/>
+      </c>
+      <c r="F35" s="10">
+        <f>D35-E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="28" t="inlineStr"/>
+      <c r="H35">
+        <f>IF(ROUND(F35,2)=0,"Settled",IF(ROUND(F35,2)&lt;0,"Overpaid","Outstanding"))</f>
         <v/>
       </c>
     </row>
@@ -6686,6 +6768,14 @@
         <f>SUM(D27:D35)</f>
         <v/>
       </c>
+      <c r="E36" s="12">
+        <f>SUM(E27:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="12">
+        <f>SUM(F27:F35)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -6701,25 +6791,33 @@
         </is>
       </c>
       <c r="B38" s="10">
-        <f>TQ_Income-IFERROR(INDEX(Costs_PartyTotals, MATCH(A38, Costs_PartyHeaders, 0)),0)</f>
-        <v/>
-      </c>
-      <c r="C38" s="24" t="inlineStr">
+        <f>TQ_Income</f>
+        <v/>
+      </c>
+      <c r="C38" s="10">
+        <f>IFERROR(INDEX(Costs_PartyTotals, MATCH(A38, Costs_PartyHeaders, 0)),0)</f>
+        <v/>
+      </c>
+      <c r="D38" s="10">
+        <f>B38-C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="24" t="inlineStr">
+      <c r="F38" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>External — TruQuant's 18% comes upstream of this pool. Their share of TQ/Armada costs is also paid externally.</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>External</t>
         </is>

</xml_diff>